<commit_message>
change endpoint qr scanner and update agents
</commit_message>
<xml_diff>
--- a/collections/test_script.xlsx
+++ b/collections/test_script.xlsx
@@ -576,8 +576,9 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155007-PJDLFV
-ktp: 7183707084435907</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105237-MROZSE
+ktp: 5174915957365173
+</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -612,7 +613,7 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -660,8 +661,9 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155007-ZIPIBD
-ktp: 3717373831486270</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-PZWTYH
+ktp: 9509999358932309
+</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -689,7 +691,7 @@
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -736,8 +738,9 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155007-WTRSMF
-ktp: 8563590623948738</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-COKQRZ
+ktp: 6054880184960160
+</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -765,7 +768,7 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -813,8 +816,9 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155008-EUAZNH
-ktp: 8775136867712021</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
+ktp: 5298525130907928
+</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -849,7 +853,7 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -897,7 +901,8 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>ktp: 7777859632741843</t>
+          <t xml:space="preserve">ktp: 8413190096541501
+</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -932,7 +937,7 @@
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -980,9 +985,10 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155008-EUAZNH
-ktp: 8775136867712021
-nomor_loan: LN-521629</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
+ktp: 5298525130907928
+nomor_loan: LN-912030
+</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1010,7 +1016,7 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1058,10 +1064,11 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155008-EUAZNH
-ktp: 8775136867712021
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
+ktp: 5298525130907928
 nomor_transaksi: TRX-INVALID
-nomor_loan: LN-904725</t>
+nomor_loan: LN-299101
+</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1089,7 +1096,7 @@
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1137,9 +1144,10 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155008-EUAZNH
-ktp: 8775136867712021
-nomor_loan: LN-521629</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
+ktp: 5298525130907928
+nomor_loan: LN-912030
+</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1167,7 +1175,7 @@
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1215,9 +1223,10 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155008-EUAZNH
-ktp: 8775136867712021
-nomor_loan: LN-521629</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
+ktp: 5298525130907928
+nomor_loan: LN-912030
+</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1245,7 +1254,7 @@
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1293,9 +1302,10 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155029-RMRZAF
-ktp: 3008913693916194
-nomor_loan: LN-821350</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105301-XTPATU
+ktp: 0095987701022186
+nomor_loan: LN-950205
+</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1323,7 +1333,7 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1371,19 +1381,17 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155008-APMQDG
-ktp: 8276085917676199
-nomor_loan: LN-289579</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105240-GIWJWE
+ktp: 8171418747522201
+nomor_loan: LN-906469
+</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Nominal Pembayaran tidak sesuai dengan Nominal Premi yang sebenarnya",
-  "data": {}
+          <t>1. {
+  "status": False,
+  "message": "Nominal Pembayaran tidak sesuai dengan Nominal Premi yang sebenarnya"
 }
 2. data tidak kerecord di DB</t>
         </is>
@@ -1401,7 +1409,7 @@
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1449,10 +1457,11 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155008-EUAZNH
-ktp: 8775136867712021
-nomor_loan: LN-521629
-nomor_transaksi: AKS-20260724-155007-PJDLFV</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
+ktp: 5298525130907928
+nomor_loan: LN-912030
+nomor_transaksi: AKS-20260805-105237-MROZSE
+</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1480,7 +1489,7 @@
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1528,9 +1537,10 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155218-YDAVNC
-ktp: 2973209137393974
-nomor_loan: LN-846121</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105359-OFCRJP
+ktp: 2444944593616553
+nomor_loan: LN-161604
+</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1558,7 +1568,7 @@
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1606,10 +1616,11 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155008-EUAZNH
-ktp: 8775136867712021
-nomor_loan: LN-521629
-nomor_transaksi: TRX-INVALID</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
+ktp: 5298525130907928
+nomor_loan: LN-912030
+nomor_transaksi: TRX-INVALID
+</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1637,7 +1648,7 @@
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1685,8 +1696,9 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-ICDKFY
-ktp: 6959271577423952</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-SFHJHV
+ktp: 2513878063754576
+</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1714,7 +1726,7 @@
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1762,8 +1774,9 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-THWQVZ
-ktp: 0673843225611107</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-HZCQIW
+ktp: 4369640609742162
+</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1791,7 +1804,7 @@
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1839,8 +1852,9 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-RONKVZ
-ktp: 6157610764187349</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-JOISMS
+ktp: 9476945598809031
+</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1868,7 +1882,7 @@
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1916,8 +1930,9 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-JCDOCO
-ktp: 3440903591011392</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-IOPZZU
+ktp: 8979904857489073
+</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1945,7 +1960,7 @@
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -1993,8 +2008,9 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-JNWYWW
-ktp: 8798270889520952</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-MNNGIV
+ktp: 4963441520371383
+</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2022,7 +2038,7 @@
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2070,8 +2086,9 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-ANOADI
-ktp: 8260314596608793</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-KLPJSG
+ktp: 3639323109780232
+</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2106,7 +2123,7 @@
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2172,8 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-YZCNJA</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-FJEOTM
+</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2183,7 +2201,7 @@
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2231,9 +2249,10 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-ANOADI
-ktp: 8260314596608793
-nomor_loan: LN-212953</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-KLPJSG
+ktp: 3639323109780232
+nomor_loan: LN-699824
+</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2261,7 +2280,7 @@
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2309,8 +2328,9 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-NNLNGG
-ktp: 8775136867712021</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-SGPBCG
+ktp: 5298525130907928
+</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2338,7 +2358,7 @@
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2386,8 +2406,9 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155223-HEIHIZ
-ktp: 5903607313768656</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-PCRVEZ
+ktp: 5271728830036242
+</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2415,7 +2436,7 @@
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2464,8 +2485,9 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155224-KEPTDH
-ktp: 6092838109797567</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-CWIBIS
+ktp: 3380420615960378
+</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2493,7 +2515,7 @@
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2542,8 +2564,9 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155224-WGEPOH
-ktp: 6566305679962000</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-ZVHTVX
+ktp: 0462971996804353
+</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2571,7 +2594,7 @@
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2620,8 +2643,9 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155224-VBJTXF
-ktp: 4208050334378278</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-PJJSDB
+ktp: 8199087614318990
+</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2649,7 +2673,7 @@
       </c>
       <c r="N30" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2696,8 +2720,9 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155224-IGAJCD
-ktp: 7183707084435907</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-DJWKVN
+ktp: 5174915957365173
+</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2732,7 +2757,7 @@
       </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -2782,15 +2807,91 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155224-UWNRST
-ktp: 2090599831425946
-nomor_transaksi: AKS-20260724-155224-SSIQBP
-nomor_loan: LN-439334
-nomor_transaksi: AKS-20260724-155224-OAJBSI
-nomor_transaksi: AKS-20260724-155225-QYCTJQ</t>
+          <t xml:space="preserve">[DATA UTAMA]
+KTP: 5354138452969705
+Loan: LN-970793
+PK: 26PK626523
+[TXs]
+T1: AKS-20260805-105405-KCBAMH
+T2: AKS-20260805-105405-JOOORP
+T3: AKS-20260805-105405-MGEZDQ
+T4: AKS-20260805-105405-PVTHYV
+</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Sistem mengizinkan reuse data (KTP, Loan, PK) selama pengajuan sebelumnya dibatalkan.</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="n"/>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>A2 - Submit Draft Akseptasi</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>TC-30</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Submit Draft - Tenor panjang (15 thn) usia debitur muda (20 thn)</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>1. Set usia_debitur = 20
+2. Set tenor = 180 bulan
+3. Hit endpoint Submit Draft</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105537-VZPDDU
+ktp: 1108698583370871
+nomor_loan: LN-214316
+nomor_loan: LN-912030
+</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>1. Response API:
 {
@@ -2802,73 +2903,73 @@
 2. data DB sesuai dengan request postman</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="L32" s="3" t="n"/>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr">
-        <is>
-          <t>24-Jul-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="n"/>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>TC-30</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Submit Draft - Tenor panjang (15 thn) usia debitur muda (20 thn)</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>TC-31</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Submit Draft - Tenor panjang (15 thn) batas akhir usia tepat 65 thn</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>1. Set usia_debitur = 20
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>1. Set usia_debitur = 50
 2. Set tenor = 180 bulan
 3. Hit endpoint Submit Draft</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>nomor_transaksi: AKS-20260724-155413-ECMFTQ
-ktp: 7686541390287803
-nomor_loan: LN-219225
-nomor_loan: LN-521629</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105601-FCPOVF
+ktp: 2373478682715971
+nomor_loan: LN-609691
+</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
         <is>
           <t>1. Response API:
 {
@@ -2880,83 +2981,6 @@
 2. data DB sesuai dengan request postman</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N33" s="3" t="inlineStr">
-        <is>
-          <t>24-Jul-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>A2 - Submit Draft Akseptasi</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>TC-31</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Submit Draft - Tenor panjang (15 thn) batas akhir usia tepat 65 thn</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>1. Set usia_debitur = 50
-2. Set tenor = 180 bulan
-3. Hit endpoint Submit Draft</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>nomor_transaksi: AKS-20260729-135157-SNKSTB
-ktp: 4485032489955195
-nomor_loan: LN-813603</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Notifikasi pembayaran berhasil diterima.",
-  "data": {}
-}
-2. data DB sesuai dengan request postman</t>
-        </is>
-      </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
@@ -2970,7 +2994,7 @@
       </c>
       <c r="N34" s="3" t="inlineStr">
         <is>
-          <t>29-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -3017,8 +3041,9 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155723-FROZCE
-ktp: 0163395304719223</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105611-IORXQX
+ktp: 8237766958960919
+</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3053,7 +3078,7 @@
       </c>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -3100,8 +3125,9 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155723-FHZPOD
-ktp: 6833669482568278</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105611-KDTMPV
+ktp: 8565889864602962
+</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3129,7 +3155,7 @@
       </c>
       <c r="N36" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -3176,8 +3202,9 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155723-FNFLZI
-ktp: 7127797096995542</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105611-TCYZHA
+ktp: 8786161155312102
+</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3205,7 +3232,7 @@
       </c>
       <c r="N37" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -3252,8 +3279,9 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260724-155723-RFLYKY
-ktp: 5562073387265097</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105611-WOCTPX
+ktp: 3600462519361894
+</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3281,7 +3309,7 @@
       </c>
       <c r="N38" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3357,8 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>ktp: 4812727259711769</t>
+          <t xml:space="preserve">ktp: 9410737665944263
+</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3364,7 +3393,7 @@
       </c>
       <c r="N39" s="3" t="inlineStr">
         <is>
-          <t>24-Jul-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update all flow and fixed
</commit_message>
<xml_diff>
--- a/collections/test_script.xlsx
+++ b/collections/test_script.xlsx
@@ -576,9 +576,8 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105237-MROZSE
-ktp: 5174915957365173
-</t>
+          <t>nomor_transaksi: AKS-20260805-165651-ZEPCCN
+ktp: 9264448493996559</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -613,7 +612,7 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -661,9 +660,8 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-PZWTYH
-ktp: 9509999358932309
-</t>
+          <t>nomor_transaksi: AKS-20260805-165651-TCZCCO
+ktp: 3616216676505898</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -691,7 +689,7 @@
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -738,9 +736,8 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-COKQRZ
-ktp: 6054880184960160
-</t>
+          <t>nomor_transaksi: AKS-20260805-165651-RVGMXL
+ktp: 7691967752283707</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -768,7 +765,7 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -816,9 +813,8 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
-ktp: 5298525130907928
-</t>
+          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
+ktp: 9041010648016044</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -853,7 +849,7 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -901,8 +897,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ktp: 8413190096541501
-</t>
+          <t>ktp: 1204739608533995</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -937,7 +932,7 @@
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -985,10 +980,9 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
-ktp: 5298525130907928
-nomor_loan: LN-912030
-</t>
+          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
+ktp: 9041010648016044
+nomor_loan: LN-912498</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1016,7 +1010,7 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1064,11 +1058,10 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
-ktp: 5298525130907928
+          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
+ktp: 9041010648016044
 nomor_transaksi: TRX-INVALID
-nomor_loan: LN-299101
-</t>
+nomor_loan: LN-222574</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1096,7 +1089,7 @@
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1144,10 +1137,9 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
-ktp: 5298525130907928
-nomor_loan: LN-912030
-</t>
+          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
+ktp: 9041010648016044
+nomor_loan: LN-912498</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1175,7 +1167,7 @@
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1223,10 +1215,9 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
-ktp: 5298525130907928
-nomor_loan: LN-912030
-</t>
+          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
+ktp: 9041010648016044
+nomor_loan: LN-912498</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1254,7 +1245,7 @@
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1302,10 +1293,9 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105301-XTPATU
-ktp: 0095987701022186
-nomor_loan: LN-950205
-</t>
+          <t>nomor_transaksi: AKS-20260805-165712-SARPWX
+ktp: 2035660357005205
+nomor_loan: LN-575441</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1333,7 +1323,7 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1381,17 +1371,19 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105240-GIWJWE
-ktp: 8171418747522201
-nomor_loan: LN-906469
-</t>
+          <t>nomor_transaksi: AKS-20260805-165652-RYURYD
+ktp: 4832932327499290
+nomor_loan: LN-045059</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>1. {
-  "status": False,
-  "message": "Nominal Pembayaran tidak sesuai dengan Nominal Premi yang sebenarnya"
+          <t>1. Response API:
+{
+  "status_code": 422,
+  "error": true,
+  "message": "Nominal Pembayaran tidak sesuai dengan Nominal Premi yang sebenarnya",
+  "data": {}
 }
 2. data tidak kerecord di DB</t>
         </is>
@@ -1409,7 +1401,7 @@
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1457,11 +1449,10 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
-ktp: 5298525130907928
-nomor_loan: LN-912030
-nomor_transaksi: AKS-20260805-105237-MROZSE
-</t>
+          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
+ktp: 9041010648016044
+nomor_loan: LN-912498
+nomor_transaksi: AKS-20260805-165651-ZEPCCN</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1489,7 +1480,7 @@
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1537,10 +1528,9 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105359-OFCRJP
-ktp: 2444944593616553
-nomor_loan: LN-161604
-</t>
+          <t>nomor_transaksi: AKS-20260805-165901-QLEGOR
+ktp: 6790192244616911
+nomor_loan: LN-056823</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1568,7 +1558,7 @@
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1616,11 +1606,10 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105239-DUOLOS
-ktp: 5298525130907928
-nomor_loan: LN-912030
-nomor_transaksi: TRX-INVALID
-</t>
+          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
+ktp: 9041010648016044
+nomor_loan: LN-912498
+nomor_transaksi: TRX-INVALID</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1648,7 +1637,7 @@
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1696,16 +1685,15 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-SFHJHV
-ktp: 2513878063754576
-</t>
+          <t>nomor_transaksi: AKS-20260805-165907-KQOFFH
+ktp: 1843914928051234</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
           <t>1. Response API:
 {
-  "timestamp": "2026-07-24T08:52:23.257Z",
+  "timestamp": "2026-08-05T09:59:07.590Z",
   "status": 400,
   "error": "Bad Request",
   "path": "/akseptasi/draft/submit"
@@ -1726,7 +1714,7 @@
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1774,9 +1762,8 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-HZCQIW
-ktp: 4369640609742162
-</t>
+          <t>nomor_transaksi: AKS-20260805-165907-TODOSG
+ktp: 2905571356950106</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1804,7 +1791,7 @@
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1852,9 +1839,8 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-JOISMS
-ktp: 9476945598809031
-</t>
+          <t>nomor_transaksi: AKS-20260805-165907-BNVZQT
+ktp: 6358019105513930</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1882,7 +1868,7 @@
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -1930,9 +1916,8 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-IOPZZU
-ktp: 8979904857489073
-</t>
+          <t>nomor_transaksi: AKS-20260805-165907-XBHUGL
+ktp: 2299982995775066</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1960,7 +1945,7 @@
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2008,9 +1993,8 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105403-MNNGIV
-ktp: 4963441520371383
-</t>
+          <t>nomor_transaksi: AKS-20260805-165907-SFHHJR
+ktp: 0816594951953397</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2038,7 +2022,7 @@
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2086,9 +2070,8 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-KLPJSG
-ktp: 3639323109780232
-</t>
+          <t>nomor_transaksi: AKS-20260805-165907-XKNAVP
+ktp: 0221219577889999</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2123,7 +2106,7 @@
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2172,8 +2155,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-FJEOTM
-</t>
+          <t>nomor_transaksi: AKS-20260805-165908-CNZXSC</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2201,7 +2183,7 @@
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2249,10 +2231,9 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-KLPJSG
-ktp: 3639323109780232
-nomor_loan: LN-699824
-</t>
+          <t>nomor_transaksi: AKS-20260805-165907-XKNAVP
+ktp: 0221219577889999
+nomor_loan: LN-061962</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2280,7 +2261,7 @@
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2328,9 +2309,8 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-SGPBCG
-ktp: 5298525130907928
-</t>
+          <t>nomor_transaksi: AKS-20260805-165908-QVDCVW
+ktp: 9041010648016044</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2358,7 +2338,7 @@
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2406,9 +2386,8 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-PCRVEZ
-ktp: 5271728830036242
-</t>
+          <t>nomor_transaksi: AKS-20260805-165908-KYEPBM
+ktp: 1355240540305847</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2436,7 +2415,7 @@
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2485,9 +2464,8 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-CWIBIS
-ktp: 3380420615960378
-</t>
+          <t>nomor_transaksi: AKS-20260805-165908-TFKVWP
+ktp: 1052500096015916</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2515,7 +2493,7 @@
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2564,9 +2542,8 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-ZVHTVX
-ktp: 0462971996804353
-</t>
+          <t>nomor_transaksi: AKS-20260805-165908-CAKMGG
+ktp: 8186499348919394</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2594,7 +2571,7 @@
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2643,9 +2620,8 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-PJJSDB
-ktp: 8199087614318990
-</t>
+          <t>nomor_transaksi: AKS-20260805-165908-TAQMCF
+ktp: 5944358434828145</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2673,7 +2649,7 @@
       </c>
       <c r="N30" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2720,9 +2696,8 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105404-DJWKVN
-ktp: 5174915957365173
-</t>
+          <t>nomor_transaksi: AKS-20260805-165908-ERLVWS
+ktp: 9264448493996559</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2757,7 +2732,7 @@
       </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -2807,91 +2782,15 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">[DATA UTAMA]
-KTP: 5354138452969705
-Loan: LN-970793
-PK: 26PK626523
-[TXs]
-T1: AKS-20260805-105405-KCBAMH
-T2: AKS-20260805-105405-JOOORP
-T3: AKS-20260805-105405-MGEZDQ
-T4: AKS-20260805-105405-PVTHYV
-</t>
+          <t>nomor_transaksi: AKS-20260805-165908-XSRKDH
+ktp: 5615733978166312
+nomor_transaksi: AKS-20260805-165909-WWNIJF
+nomor_loan: LN-653977
+nomor_transaksi: AKS-20260805-165909-XBDHMW
+nomor_transaksi: AKS-20260805-165909-OQHOTS</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>Sistem mengizinkan reuse data (KTP, Loan, PK) selama pengajuan sebelumnya dibatalkan.</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="L32" s="3" t="n"/>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr">
-        <is>
-          <t>05/08/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>A2 - Submit Draft Akseptasi</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>TC-30</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Submit Draft - Tenor panjang (15 thn) usia debitur muda (20 thn)</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>1. Set usia_debitur = 20
-2. Set tenor = 180 bulan
-3. Hit endpoint Submit Draft</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105537-VZPDDU
-ktp: 1108698583370871
-nomor_loan: LN-214316
-nomor_loan: LN-912030
-</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>1. Response API:
 {
@@ -2903,73 +2802,73 @@
 2. data DB sesuai dengan request postman</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N33" s="3" t="inlineStr">
-        <is>
-          <t>05/08/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="n"/>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>05-Aug-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>TC-31</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Submit Draft - Tenor panjang (15 thn) batas akhir usia tepat 65 thn</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>TC-30</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Submit Draft - Tenor panjang (15 thn) usia debitur muda (20 thn)</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>1. Set usia_debitur = 50
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>1. Set usia_debitur = 20
 2. Set tenor = 180 bulan
 3. Hit endpoint Submit Draft</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105601-FCPOVF
-ktp: 2373478682715971
-nomor_loan: LN-609691
-</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>nomor_transaksi: AKS-20260805-170117-RRBVBO
+ktp: 8741155139641624
+nomor_loan: LN-446135
+nomor_loan: LN-912498</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>1. Response API:
 {
@@ -2981,6 +2880,83 @@
 2. data DB sesuai dengan request postman</t>
         </is>
       </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="n"/>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>05-Aug-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>A2 - Submit Draft Akseptasi</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>TC-31</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Submit Draft - Tenor panjang (15 thn) batas akhir usia tepat 65 thn</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>1. Set usia_debitur = 50
+2. Set tenor = 180 bulan
+3. Hit endpoint Submit Draft</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>nomor_transaksi: AKS-20260805-170144-ZAUERC
+ktp: 5036032729651061
+nomor_loan: LN-524785</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>1. Response API:
+{
+  "status_code": 200,
+  "error": false,
+  "message": "Notifikasi pembayaran berhasil diterima.",
+  "data": {}
+}
+2. data DB sesuai dengan request postman</t>
+        </is>
+      </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
@@ -2994,7 +2970,7 @@
       </c>
       <c r="N34" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -3041,9 +3017,8 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105611-IORXQX
-ktp: 8237766958960919
-</t>
+          <t>nomor_transaksi: AKS-20260805-170454-AZAAGP
+ktp: 1833572943601969</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3078,7 +3053,7 @@
       </c>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -3125,9 +3100,8 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105611-KDTMPV
-ktp: 8565889864602962
-</t>
+          <t>nomor_transaksi: AKS-20260805-170455-EYKZWH
+ktp: 4925633547127541</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3155,7 +3129,7 @@
       </c>
       <c r="N36" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -3202,9 +3176,8 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105611-TCYZHA
-ktp: 8786161155312102
-</t>
+          <t>nomor_transaksi: AKS-20260805-170455-JPMPYU
+ktp: 2267557116949113</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3232,7 +3205,7 @@
       </c>
       <c r="N37" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -3279,9 +3252,8 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260805-105611-WOCTPX
-ktp: 3600462519361894
-</t>
+          <t>nomor_transaksi: AKS-20260805-170455-BGIPMZ
+ktp: 0788340952015482</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3309,7 +3281,7 @@
       </c>
       <c r="N38" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -3357,8 +3329,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ktp: 9410737665944263
-</t>
+          <t>ktp: 9769052535888946</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3393,7 +3364,7 @@
       </c>
       <c r="N39" s="3" t="inlineStr">
         <is>
-          <t>05/08/2026</t>
+          <t>05-Aug-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update flow business integrate to test script
</commit_message>
<xml_diff>
--- a/collections/test_script.xlsx
+++ b/collections/test_script.xlsx
@@ -455,7 +455,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Test Script SIT - PENGEMBANGAN KMG JATIM GEN 2</t>
+          <t>Test Script - TESTING (TESTING)</t>
         </is>
       </c>
     </row>
@@ -576,8 +576,9 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-ZEPCCN
-ktp: 9264448493996559</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135109-HIUNBL
+ktp: 2684298875624968
+</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -612,7 +613,7 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -660,8 +661,9 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-TCZCCO
-ktp: 3616216676505898</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-BGFLVJ
+ktp: 7395033966692873
+</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -689,7 +691,7 @@
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -736,8 +738,9 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-RVGMXL
-ktp: 7691967752283707</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-STXPJA
+ktp: 6309371396477808
+</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -765,7 +768,7 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -813,8 +816,9 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
-ktp: 9041010648016044</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
+ktp: 9788115849876051
+</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -849,7 +853,7 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -897,7 +901,8 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>ktp: 1204739608533995</t>
+          <t xml:space="preserve">ktp: 4863466280264534
+</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -932,7 +937,7 @@
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -980,9 +985,10 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
-ktp: 9041010648016044
-nomor_loan: LN-912498</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
+ktp: 9788115849876051
+nomor_loan: LN-230392
+</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1010,7 +1016,7 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1058,10 +1064,11 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
-ktp: 9041010648016044
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
+ktp: 9788115849876051
 nomor_transaksi: TRX-INVALID
-nomor_loan: LN-222574</t>
+nomor_loan: LN-368707
+</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1089,7 +1096,7 @@
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1137,9 +1144,10 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
-ktp: 9041010648016044
-nomor_loan: LN-912498</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
+ktp: 9788115849876051
+nomor_loan: LN-230392
+</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1167,7 +1175,7 @@
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1215,9 +1223,10 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
-ktp: 9041010648016044
-nomor_loan: LN-912498</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
+ktp: 9788115849876051
+nomor_loan: LN-230392
+</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1245,7 +1254,7 @@
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1293,9 +1302,10 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165712-SARPWX
-ktp: 2035660357005205
-nomor_loan: LN-575441</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135133-XPXVWC
+ktp: 6593313455567324
+nomor_loan: LN-210110
+</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1323,7 +1333,7 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1371,19 +1381,17 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165652-RYURYD
-ktp: 4832932327499290
-nomor_loan: LN-045059</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135112-YHZZPT
+ktp: 2449145585016433
+nomor_loan: LN-596459
+</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Nominal Pembayaran tidak sesuai dengan Nominal Premi yang sebenarnya",
-  "data": {}
+          <t>1. {
+  "status": False,
+  "message": "Nominal Pembayaran tidak sesuai dengan Nominal Premi yang sebenarnya"
 }
 2. data tidak kerecord di DB</t>
         </is>
@@ -1401,7 +1409,7 @@
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1449,10 +1457,11 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
-ktp: 9041010648016044
-nomor_loan: LN-912498
-nomor_transaksi: AKS-20260805-165651-ZEPCCN</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
+ktp: 9788115849876051
+nomor_loan: LN-230392
+nomor_transaksi: AKS-20260807-135109-HIUNBL
+</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1480,7 +1489,7 @@
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1528,9 +1537,10 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165901-QLEGOR
-ktp: 6790192244616911
-nomor_loan: LN-056823</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135349-VAIAVM
+ktp: 5527479402189147
+nomor_loan: LN-472214
+</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1558,7 +1568,7 @@
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1606,10 +1616,11 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165651-ILPBMY
-ktp: 9041010648016044
-nomor_loan: LN-912498
-nomor_transaksi: TRX-INVALID</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
+ktp: 9788115849876051
+nomor_loan: LN-230392
+nomor_transaksi: TRX-INVALID
+</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1637,7 +1648,7 @@
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1685,8 +1696,9 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165907-KQOFFH
-ktp: 1843914928051234</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135353-VLNLNQ
+ktp: 9181813928208282
+</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1714,7 +1726,7 @@
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1762,8 +1774,9 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165907-TODOSG
-ktp: 2905571356950106</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-TWETXJ
+ktp: 6625810764947677
+</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1791,7 +1804,7 @@
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1839,8 +1852,9 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165907-BNVZQT
-ktp: 6358019105513930</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-ICYPGO
+ktp: 4613669445055595
+</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1868,7 +1882,7 @@
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1916,8 +1930,9 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165907-XBHUGL
-ktp: 2299982995775066</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-SUVHGB
+ktp: 4892014647387048
+</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1945,7 +1960,7 @@
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -1993,8 +2008,9 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165907-SFHHJR
-ktp: 0816594951953397</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-KRHQEZ
+ktp: 8782312054560221
+</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2022,7 +2038,7 @@
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2070,8 +2086,9 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165907-XKNAVP
-ktp: 0221219577889999</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-CFUQNV
+ktp: 1220519002834480
+</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2106,7 +2123,7 @@
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2172,8 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165908-CNZXSC</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-QQBFLR
+</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2183,7 +2201,7 @@
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2231,9 +2249,10 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165907-XKNAVP
-ktp: 0221219577889999
-nomor_loan: LN-061962</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-CFUQNV
+ktp: 1220519002834480
+nomor_loan: LN-016902
+</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2261,7 +2280,7 @@
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2309,8 +2328,9 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165908-QVDCVW
-ktp: 9041010648016044</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-EAQPUY
+ktp: 9788115849876051
+</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2338,7 +2358,7 @@
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2386,8 +2406,9 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165908-KYEPBM
-ktp: 1355240540305847</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-KWGYMU
+ktp: 9541658848961073
+</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2415,7 +2436,7 @@
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2464,8 +2485,9 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165908-TFKVWP
-ktp: 1052500096015916</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-TYLUCP
+ktp: 9406718152857607
+</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2493,7 +2515,7 @@
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2542,8 +2564,9 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165908-CAKMGG
-ktp: 8186499348919394</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-NEOEEK
+ktp: 7917462899997153
+</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2571,7 +2594,7 @@
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2620,8 +2643,9 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165908-TAQMCF
-ktp: 5944358434828145</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-NNTBTX
+ktp: 6163685265773691
+</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2649,7 +2673,7 @@
       </c>
       <c r="N30" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2696,8 +2720,9 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165908-ERLVWS
-ktp: 9264448493996559</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-LEOTWX
+ktp: 2684298875624968
+</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2732,7 +2757,7 @@
       </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -2782,15 +2807,91 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-165908-XSRKDH
-ktp: 5615733978166312
-nomor_transaksi: AKS-20260805-165909-WWNIJF
-nomor_loan: LN-653977
-nomor_transaksi: AKS-20260805-165909-XBDHMW
-nomor_transaksi: AKS-20260805-165909-OQHOTS</t>
+          <t xml:space="preserve">[DATA UTAMA]
+KTP: 4342581324629421
+Loan: LN-937289
+PK: 26PK144985
+[TXs]
+T1: AKS-20260807-135355-YJXXNB
+T2: AKS-20260807-135355-REBJBE
+T3: AKS-20260807-135355-QWSXHZ
+T4: AKS-20260807-135355-VFBBFL
+</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Sistem mengizinkan reuse data (KTP, Loan, PK) selama pengajuan sebelumnya dibatalkan.</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="n"/>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>A2 - Submit Draft Akseptasi</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>TC-30</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Submit Draft - Tenor panjang (15 thn) usia debitur muda (20 thn)</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>1. Set usia_debitur = 20
+2. Set tenor = 180 bulan
+3. Hit endpoint Submit Draft</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135556-DBTUUJ
+ktp: 5773972188662761
+nomor_loan: LN-980324
+nomor_loan: LN-230392
+</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>1. Response API:
 {
@@ -2802,73 +2903,73 @@
 2. data DB sesuai dengan request postman</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="L32" s="3" t="n"/>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr">
-        <is>
-          <t>05-Aug-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="n"/>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>TC-30</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Submit Draft - Tenor panjang (15 thn) usia debitur muda (20 thn)</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>TC-31</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Submit Draft - Tenor panjang (15 thn) batas akhir usia tepat 65 thn</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>1. Set usia_debitur = 20
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>1. Set usia_debitur = 50
 2. Set tenor = 180 bulan
 3. Hit endpoint Submit Draft</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>nomor_transaksi: AKS-20260805-170117-RRBVBO
-ktp: 8741155139641624
-nomor_loan: LN-446135
-nomor_loan: LN-912498</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135621-HBWZEC
+ktp: 1391133790621687
+nomor_loan: LN-049771
+</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
         <is>
           <t>1. Response API:
 {
@@ -2880,83 +2981,6 @@
 2. data DB sesuai dengan request postman</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N33" s="3" t="inlineStr">
-        <is>
-          <t>05-Aug-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>A2 - Submit Draft Akseptasi</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>TC-31</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Submit Draft - Tenor panjang (15 thn) batas akhir usia tepat 65 thn</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>1. Set usia_debitur = 50
-2. Set tenor = 180 bulan
-3. Hit endpoint Submit Draft</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>nomor_transaksi: AKS-20260805-170144-ZAUERC
-ktp: 5036032729651061
-nomor_loan: LN-524785</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Notifikasi pembayaran berhasil diterima.",
-  "data": {}
-}
-2. data DB sesuai dengan request postman</t>
-        </is>
-      </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
@@ -2970,7 +2994,7 @@
       </c>
       <c r="N34" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -3017,8 +3041,9 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-170454-AZAAGP
-ktp: 1833572943601969</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135816-BUPXTK
+ktp: 0382848240684456
+</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3053,7 +3078,7 @@
       </c>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -3100,8 +3125,9 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-170455-EYKZWH
-ktp: 4925633547127541</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135816-PQKNJV
+ktp: 3362076993722731
+</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3129,7 +3155,7 @@
       </c>
       <c r="N36" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -3176,8 +3202,9 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-170455-JPMPYU
-ktp: 2267557116949113</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135817-RSKZPZ
+ktp: 0188868782533446
+</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3205,7 +3232,7 @@
       </c>
       <c r="N37" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -3252,8 +3279,9 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>nomor_transaksi: AKS-20260805-170455-BGIPMZ
-ktp: 0788340952015482</t>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135817-ZPRXZY
+ktp: 7735628363597715
+</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3281,7 +3309,7 @@
       </c>
       <c r="N38" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3357,8 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>ktp: 9769052535888946</t>
+          <t xml:space="preserve">ktp: 5490546700588970
+</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3364,7 +3393,7 @@
       </c>
       <c r="N39" s="3" t="inlineStr">
         <is>
-          <t>05-Aug-2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
modified structure and result in report
</commit_message>
<xml_diff>
--- a/collections/test_script.xlsx
+++ b/collections/test_script.xlsx
@@ -576,28 +576,16 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135109-HIUNBL
-ktp: 2684298875624968
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094853-WXZGIP
+ktp: 6621997483706595
 </t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Draft akseptasi berhasil diterima.",
-  "data": {
-    "medical_code": "CAC",
-    "premi": 72500.0,
-    "rate": 0.145,
-    "akumulasi": false,
-    "nilai_akumulasi": 0,
-    "list_dokumen_underwriting": []
-  }
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -613,7 +601,7 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -661,21 +649,15 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-BGFLVJ
-ktp: 7395033966692873
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-RHYKMR
+ktp: 7061651407279214
 </t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Uang pertanggungan tidak boleh kosong dan harus lebih besar dari 0",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -691,7 +673,7 @@
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -738,21 +720,15 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-STXPJA
-ktp: 6309371396477808
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-VVIKIN
+ktp: 3169545050669331
 </t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Kode Unit Kerja tidak ditemukan",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -768,7 +744,7 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -816,28 +792,16 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
-ktp: 9788115849876051
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
+ktp: 0687495697403336
 </t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Draft akseptasi berhasil diterima.",
-  "data": {
-    "medical_code": "CAC",
-    "premi": 72500.0,
-    "rate": 0.145,
-    "akumulasi": false,
-    "nilai_akumulasi": 0,
-    "list_dokumen_underwriting": []
-  }
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -853,7 +817,7 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -901,27 +865,15 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ktp: 4863466280264534
+          <t xml:space="preserve">ktp: 3118541964223781
 </t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "data": {
-    "akumulasi": false,
-    "list_dokumen_underwriting": [],
-    "medical_code": "CAC",
-    "nilai_akumulasi": 0.0,
-    "premi": 362500.0,
-    "rate": 0.725
-  },
-  "error": false,
-  "message": "Kalkulasi Premi Berhasil",
-  "status_code": 200
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -937,7 +889,7 @@
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -985,22 +937,17 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
-ktp: 9788115849876051
-nomor_loan: LN-230392
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
+ktp: 0687495697403336
+nomor_loan: LN-441777
 </t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Inquiry nomor loan berhasil diterima.",
-  "data": {}
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -1016,7 +963,7 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1064,23 +1011,17 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
-ktp: 9788115849876051
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
+ktp: 0687495697403336
 nomor_transaksi: TRX-INVALID
-nomor_loan: LN-368707
+nomor_loan: LN-072135
 </t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Data pengajuan akseptasi dengan nomor transaksi TRX-INVALID tidak ditemukan",
-  "data": {}
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -1096,7 +1037,7 @@
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1144,22 +1085,17 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
-ktp: 9788115849876051
-nomor_loan: LN-230392
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
+ktp: 0687495697403336
+nomor_loan: LN-441777
 </t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Otorisasi berhasil diterima.",
-  "data": {}
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -1175,7 +1111,7 @@
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1223,22 +1159,16 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
-ktp: 9788115849876051
-nomor_loan: LN-230392
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
+ktp: 0687495697403336
+nomor_loan: LN-441777
 </t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Otorisasi berhasil diterima.",
-  "data": {}
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -1254,7 +1184,7 @@
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1302,22 +1232,17 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135133-XPXVWC
-ktp: 6593313455567324
-nomor_loan: LN-210110
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094920-KBWKJB
+ktp: 2928301182700269
+nomor_loan: LN-116216
 </t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Notifikasi pembayaran berhasil diterima.",
-  "data": {}
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -1333,7 +1258,7 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1381,19 +1306,17 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135112-YHZZPT
-ktp: 2449145585016433
-nomor_loan: LN-596459
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094858-UEQTGC
+ktp: 6913777406851537
+nomor_loan: LN-973526
 </t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>1. {
-  "status": False,
-  "message": "Nominal Pembayaran tidak sesuai dengan Nominal Premi yang sebenarnya"
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request karena nominal pembayaran salah.
+2. Response menampilkan pesan: 'Nominal Pembayaran tidak sesuai dengan Nominal Premi yang sebenarnya'.
+3. Data pembayaran tidak ter-record di Database.</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -1409,7 +1332,7 @@
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1457,23 +1380,18 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
-ktp: 9788115849876051
-nomor_loan: LN-230392
-nomor_transaksi: AKS-20260807-135109-HIUNBL
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
+ktp: 0687495697403336
+nomor_loan: LN-441777
+nomor_transaksi: AKS-20260810-094853-WXZGIP
 </t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Pembatalan draft berhasil diterima.",
-  "data": {}
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -1489,7 +1407,7 @@
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1537,22 +1455,16 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135349-VAIAVM
-ktp: 5527479402189147
-nomor_loan: LN-472214
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095125-CCBTFA
+ktp: 2640414536169631
+nomor_loan: LN-538320
 </t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Pengajuan Pembatalan Tidak dapat diproses, Status Pertanggungan Aktif",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -1568,7 +1480,7 @@
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1616,23 +1528,17 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135110-HEOPXT
-ktp: 9788115849876051
-nomor_loan: LN-230392
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
+ktp: 0687495697403336
+nomor_loan: LN-441777
 nomor_transaksi: TRX-INVALID
 </t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Data pengajuan tidak ditemukan",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -1648,7 +1554,7 @@
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1696,21 +1602,15 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135353-VLNLNQ
-ktp: 9181813928208282
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-TSWFWH
+ktp: 8543131055449504
 </t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "timestamp": "2026-08-05T09:59:07.590Z",
-  "status": 400,
-  "error": "Bad Request",
-  "path": "/akseptasi/draft/submit"
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -1726,7 +1626,7 @@
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1774,21 +1674,15 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-TWETXJ
-ktp: 6625810764947677
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-YZBRWO
+ktp: 0240573155028148
 </t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Usia ditambah tenor tidak boleh lebih dari 65 tahun",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -1804,7 +1698,7 @@
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1852,21 +1746,15 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-ICYPGO
-ktp: 4613669445055595
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-IHKIZS
+ktp: 8488796958635494
 </t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Kode Pos tidak ditemukan",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -1882,7 +1770,7 @@
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -1930,21 +1818,15 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-SUVHGB
-ktp: 4892014647387048
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-EPSIPR
+ktp: 7883901891480519
 </t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Usia ditambah tenor tidak boleh lebih dari 65 tahun",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -1960,7 +1842,7 @@
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2008,21 +1890,15 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-KRHQEZ
-ktp: 8782312054560221
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-AOVQLY
+ktp: 2656511007919077
 </t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Jumlah tenor tidak sesuai dengan selisih tanggal realisasi terhadap tanggal akhir asuransi",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -2038,7 +1914,7 @@
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2086,28 +1962,16 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-CFUQNV
-ktp: 1220519002834480
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-HNGUKI
+ktp: 4288329925398444
 </t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Draft akseptasi berhasil diterima.",
-  "data": {
-    "medical_code": "CAC",
-    "premi": 72500.0,
-    "rate": 0.145,
-    "akumulasi": false,
-    "nilai_akumulasi": 0,
-    "list_dokumen_underwriting": []
-  }
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -2123,7 +1987,7 @@
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2172,20 +2036,14 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-QQBFLR
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095157-FDVATC
 </t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "KTP tidak boleh kosong",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -2201,7 +2059,7 @@
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2249,22 +2107,16 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-CFUQNV
-ktp: 1220519002834480
-nomor_loan: LN-016902
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-HNGUKI
+ktp: 4288329925398444
+nomor_loan: LN-952100
 </t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Tanggal akad tidak boleh melebihi tanggal rencana realisasi",
-  "data": {}
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -2280,7 +2132,7 @@
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2328,21 +2180,15 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-EAQPUY
-ktp: 9788115849876051
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095157-JCUEMP
+ktp: 0687495697403336
 </t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Pengajuan tidak dapat diproses, NIK sudah terdaftar",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -2358,7 +2204,7 @@
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2406,21 +2252,15 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-KWGYMU
-ktp: 9541658848961073
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095205-NVROFY
+ktp: 1725458943535859
 </t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Usia pada saat realisasi harus lebih dari 18 tahun (minimal 18 tahun 1 hari)",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -2436,7 +2276,7 @@
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2485,21 +2325,15 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-TYLUCP
-ktp: 9406718152857607
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095206-SWUPPG
+ktp: 7933509472397987
 </t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Usia pada saat realisasi harus lebih dari 18 tahun (minimal 18 tahun 1 hari)",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -2515,7 +2349,7 @@
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2564,21 +2398,15 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-NEOEEK
-ktp: 7917462899997153
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095206-ELFQJA
+ktp: 8630458139439239
 </t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Usia ditambah tenor tidak boleh lebih dari 65 tahun",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -2594,7 +2422,7 @@
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2643,21 +2471,15 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-NNTBTX
-ktp: 6163685265773691
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095206-NUKGML
+ktp: 4201277434371275
 </t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Usia ditambah tenor tidak boleh lebih dari 65 tahun",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
@@ -2673,7 +2495,7 @@
       </c>
       <c r="N30" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2720,33 +2542,21 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135354-LEOTWX
-ktp: 2684298875624968
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-095206-TMEZHX
+ktp: 6621997483706595
 </t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Draft akseptasi berhasil diterima.",
-  "data": {
-    "medical_code": "CAC",
-    "premi": 72500.0,
-    "rate": 0.145,
-    "akumulasi": true,
-    "nilai_akumulasi": 50000000,
-    "list_dokumen_underwriting": []
-  }
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="L31" s="3" t="n"/>
@@ -2757,7 +2567,7 @@
       </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2808,14 +2618,14 @@
       <c r="I32" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">[DATA UTAMA]
-KTP: 4342581324629421
-Loan: LN-937289
-PK: 26PK144985
+KTP: 6038990022059559
+Loan: LN-119324
+PK: 26PK634907
 [TXs]
-T1: AKS-20260807-135355-YJXXNB
-T2: AKS-20260807-135355-REBJBE
-T3: AKS-20260807-135355-QWSXHZ
-T4: AKS-20260807-135355-VFBBFL
+T1: AKS-20260810-093344-WNXJIW
+T2: AKS-20260810-093344-MTBZSU
+T3: AKS-20260810-093345-IINNGQ
+T4: AKS-20260810-093345-TFZEFS
 </t>
         </is>
       </c>
@@ -2826,7 +2636,7 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="L32" s="3" t="n"/>
@@ -2837,7 +2647,7 @@
       </c>
       <c r="N32" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2884,28 +2694,23 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135556-DBTUUJ
-ktp: 5773972188662761
-nomor_loan: LN-980324
-nomor_loan: LN-230392
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-093407-SRVUEE
+ktp: 3404387391812951
+nomor_loan: LN-382229
+nomor_loan: LN-035643
 </t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Notifikasi pembayaran berhasil diterima.",
-  "data": {}
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="L33" s="3" t="n"/>
@@ -2916,7 +2721,7 @@
       </c>
       <c r="N33" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -2963,22 +2768,17 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135621-HBWZEC
-ktp: 1391133790621687
-nomor_loan: LN-049771
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-102717-RWYFZM
+ktp: 5376576102555745
+nomor_loan: LN-048388
 </t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Notifikasi pembayaran berhasil diterima.",
-  "data": {}
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
@@ -2994,7 +2794,7 @@
       </c>
       <c r="N34" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -3041,33 +2841,21 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135816-BUPXTK
-ktp: 0382848240684456
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-100018-TNTREC
+ktp: 6359327397846375
 </t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 200,
-  "error": false,
-  "message": "Draft akseptasi berhasil diterima.",
-  "data": {
-    "medical_code": "CAC",
-    "premi": 362500.0,
-    "rate": 0.725,
-    "akumulasi": false,
-    "nilai_akumulasi": 0,
-    "list_dokumen_underwriting": []
-  }
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="L35" s="3" t="n"/>
@@ -3078,7 +2866,7 @@
       </c>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -3125,26 +2913,20 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135816-PQKNJV
-ktp: 3362076993722731
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-100019-GSUROR
+ktp: 2999787370638519
 </t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Usia ditambah tenor tidak boleh lebih dari 65 tahun",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="L36" s="3" t="n"/>
@@ -3155,7 +2937,7 @@
       </c>
       <c r="N36" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -3202,26 +2984,20 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135817-RSKZPZ
-ktp: 0188868782533446
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-100019-XVOYRS
+ktp: 0136768188684338
 </t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Usia ditambah tenor tidak boleh lebih dari 65 tahun",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="L37" s="3" t="n"/>
@@ -3232,7 +3008,7 @@
       </c>
       <c r="N37" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -3279,26 +3055,20 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260807-135817-ZPRXZY
-ktp: 7735628363597715
+          <t xml:space="preserve">nomor_transaksi: AKS-20260810-100019-DGMKFO
+ktp: 8318594002702523
 </t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "status_code": 422,
-  "error": true,
-  "message": "Jumlah tenor tidak sesuai dengan selisih tanggal realisasi terhadap tanggal akhir asuransi",
-  "data": null
-}
-2. data tidak kerecord di DB</t>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="L38" s="3" t="n"/>
@@ -3309,7 +3079,7 @@
       </c>
       <c r="N38" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>
@@ -3357,27 +3127,14 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ktp: 5490546700588970
+          <t xml:space="preserve">ktp: 8217887972843606
 </t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>1. Response API:
-{
-  "data": {
-    "akumulasi": false,
-    "list_dokumen_underwriting": [],
-    "medical_code": "CAC",
-    "nilai_akumulasi": 0.0,
-    "premi": 362500.0,
-    "rate": 0.725
-  },
-  "error": false,
-  "message": "Kalkulasi Premi Berhasil",
-  "status_code": 200
-}
-2. data DB sesuai dengan request postman</t>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
@@ -3393,7 +3150,7 @@
       </c>
       <c r="N39" s="3" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add new test case multi fasilitas
</commit_message>
<xml_diff>
--- a/collections/test_script.xlsx
+++ b/collections/test_script.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,30 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="20"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00003366"/>
-        <bgColor rgb="00003366"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -56,34 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,124 +413,189 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Test Script - TESTING (TESTING)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Unnamed: 1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Unnamed: 3</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Unnamed: 4</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Unnamed: 5</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Unnamed: 6</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Unnamed: 7</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Unnamed: 8</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Unnamed: 9</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Unnamed: 10</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Unnamed: 11</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Unnamed: 12</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Unnamed: 13</t>
         </is>
       </c>
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Stream</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Nama Modul</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>TestCase-ID</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Test Case</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Jenis Test</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Pre Condition</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Nama Tester</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Tanggal Testing</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>TC-1</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Validasi sukses kalkulasi premi dengan UP 5.000.000 (Premi Dasar &lt; Batas Meterai, Admin = Batas Bawah)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit
@@ -574,72 +603,71 @@
 4. Hit Send dan check hasil response postman dan DB</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094853-WXZGIP
 ktp: 6621997483706595
 </t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>TC-2</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Submit pengajuan akseptasi dengan uang pertanggungan bernilai 0</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit
@@ -647,142 +675,140 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-RHYKMR
 ktp: 7061651407279214
 </t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>TC-3</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Submit pengajuan akseptasi menggunakan kode bank yang tidak ada di sistem mapping</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit dan Edit field kode_bank 
 3. Hit Send</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-VVIKIN
 ktp: 3169545050669331
 </t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>TC-4</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Submit pengajuan akseptasi dengan code produk yang sesuai dengan product bank</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t xml:space="preserve">[Test_Step-1] :  Buka Postman
 [Test_Step-2] :  {{TESTING_API_GATEWAY}}/akseptasi/draft/submit 
@@ -790,72 +816,71 @@
 </t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
 ktp: 0687495697403336
 </t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>A1 - Kalkulasi Premi</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>TC-5</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Hit endpoint kalkulasi premi untuk mendapatkan nilai premi secara instan dengan parameter valid</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Service API aktif dan database dalam keadaan normal.</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/calculate/premi
@@ -863,71 +888,70 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t xml:space="preserve">ktp: 3118541964223781
 </t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>A4 - Inquiry Nomor Loan</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>TC-6</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Inquiry data loan dengan menggunakan nomor transaksi draft akseptasi dan nomor rekening (loan) yang valid</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Terdapat data Draft Akseptasi yang telah sukses disubmit dan tercatat di database.</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/loan/inquiry
@@ -935,7 +959,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
 ktp: 0687495697403336
@@ -943,65 +967,64 @@
 </t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>A4 - Inquiry Nomor Loan</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>TC-7</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Mencoba inquiry data loan menggunakan nomor_transaksi fiktif yang tidak ada di database</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Terdapat data Draft Akseptasi yang telah sukses disubmit dan tercatat di database.</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/loan/inquiry
@@ -1009,7 +1032,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
 ktp: 0687495697403336
@@ -1018,64 +1041,63 @@
 </t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>A5 - Otorisasi Penyelia Bank</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>TC-8</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t xml:space="preserve">Submit status otorisasi DISETUJUI dari penyelia bank </t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Terdapat data Loan yang telah sukses melewati tahap Inquiry (A4).</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/loan/otorisasi
@@ -1083,7 +1105,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
 ktp: 0687495697403336
@@ -1091,65 +1113,64 @@
 </t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>A5 - Otorisasi Penyelia Bank</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>TC-9</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Submit status otorisasi DITOLAK karena nasabah batal kredit atau plafon final tidak disetujui</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Terdapat data Loan yang telah sukses melewati tahap Inquiry (A4).</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/loan/otorisasi
@@ -1157,7 +1178,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
 ktp: 0687495697403336
@@ -1165,64 +1186,63 @@
 </t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>A6 - Notifikasi Pembayaran Premi</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>TC-10</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Submit notifikasi pembayaran premi dengan jumlah uang yang sama persis dengan total premi (Full Payment)</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Terdapat data pengajuan yang telah mendapatkan Otorisasi (A5) dengan status DISETUJUI.</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/loan/payment
@@ -1230,7 +1250,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094920-KBWKJB
 ktp: 2928301182700269
@@ -1238,65 +1258,64 @@
 </t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>A6 - Notifikasi Pembayaran Premi</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>TC-11</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t xml:space="preserve">Submit notifikasi pembayaran premi dengan nominal yang kurang dari total tagihan premi </t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Terdapat data pengajuan yang telah mendapatkan Otorisasi (A5) dengan status DISETUJUI.</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/loan/payment
@@ -1304,7 +1323,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094858-UEQTGC
 ktp: 6913777406851537
@@ -1312,65 +1331,64 @@
 </t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>1. API menolak request karena nominal pembayaran salah.
 2. Response menampilkan pesan: 'Nominal Pembayaran tidak sesuai dengan Nominal Premi yang sebenarnya'.
 3. Data pembayaran tidak ter-record di Database.</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>A7 - Pembatalan Draft (Canceled)</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>TC-12</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Submit permintaan pembatalan draf akseptasi sebelum premi dibayarkan</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Terdapat data pengajuan aktif di database yang memenuhi syarat pembatalan.</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/canceled
@@ -1378,7 +1396,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
 ktp: 0687495697403336
@@ -1387,65 +1405,64 @@
 </t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N15" s="3" t="inlineStr">
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>A7 - Pembatalan Draft (Canceled)</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>TC-13</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>melakukan pembatalan (A7) pada nomor transaksi yang statusnya sudah POLIS_ISSUED/Terbit</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Terdapat data pengajuan aktif di database yang memenuhi syarat pembatalan.</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/canceled
@@ -1453,7 +1470,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095125-CCBTFA
 ktp: 2640414536169631
@@ -1461,64 +1478,63 @@
 </t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L16" s="3" t="n"/>
-      <c r="M16" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N16" s="3" t="inlineStr">
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>A7 - Pembatalan Draft (Canceled)</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>TC-14</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Mencoba melakukan pembatalan dengan menggunakan nomor transaksi yang tidak terdaftar</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Terdapat data pengajuan aktif di database yang memenuhi syarat pembatalan.</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/canceled
@@ -1526,7 +1542,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-094855-PKYKQL
 ktp: 0687495697403336
@@ -1535,64 +1551,63 @@
 </t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L17" s="3" t="n"/>
-      <c r="M17" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N17" s="3" t="inlineStr">
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>TC-15</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Submit pengajuan akseptasi dengan parameter 'usia' yang tidak cocok dengan hasil perhitungan 'tanggal_lahir'</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit
@@ -1600,71 +1615,70 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-TSWFWH
 ktp: 8543131055449504
 </t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N18" s="3" t="inlineStr">
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>TC-16</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Submit pengajuan dengan 'tenor' yang tidak sesuai dengan jarak antara 'tanggal_rencana_realisasi' dan 'tanggal_akhir_asuransi'</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit
@@ -1672,71 +1686,70 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-YZBRWO
 ktp: 0240573155028148
 </t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L19" s="3" t="n"/>
-      <c r="M19" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N19" s="3" t="inlineStr">
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>TC-17</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Submit pengajuan dengan 'kode_pos' berformat salah (mengandung huruf) atau kode fiktif yang tidak terdaftar di database</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit
@@ -1744,71 +1757,70 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-IHKIZS
 ktp: 8488796958635494
 </t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L20" s="3" t="n"/>
-      <c r="M20" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N20" s="3" t="inlineStr">
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>TC-18</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Submit pengajuan dimana Usia ditambah Tenor Pinjaman melebihi batas usia maksimal pertanggungan asuransi</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit
@@ -1816,71 +1828,70 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-EPSIPR
 ktp: 7883901891480519
 </t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N21" s="3" t="inlineStr">
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>TC-19</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Submit pengajuan dengan tanggal_rencana_realisasi lebih kecil dari tanggal hari ini (Backdated)</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit
@@ -1888,71 +1899,70 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-AOVQLY
 ktp: 2656511007919077
 </t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N22" s="3" t="inlineStr">
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>TC-20</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Submit pengajuan akseptasi menggunakan kode cabang bank atau kode unit kerja yang fiktif atau tidak terdaftar</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit
@@ -1960,72 +1970,71 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-HNGUKI
 ktp: 4288329925398444
 </t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N23" s="3" t="inlineStr">
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>TC-21</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Check semua Mandatory Field</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {base_url}/akseptasi/draft/submit
@@ -2034,70 +2043,69 @@
 5. Hit Send</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095157-FDVATC
 </t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="A25" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>A4 - Inquiry Nomor Loan</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>TC-22</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Hit inquiry loan ketika tanggal akad melebihi tanggal realisasi</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Terdapat data Draft Akseptasi yang telah sukses disubmit dan tercatat di database.</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST  {{TESTING_API_GATEWAY}}/akseptasi/loan/inquiry
@@ -2105,7 +2113,7 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095136-HNGUKI
 ktp: 4288329925398444
@@ -2113,64 +2121,63 @@
 </t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L25" s="3" t="n"/>
-      <c r="M25" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N25" s="3" t="inlineStr">
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
+      <c r="A26" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>TC-23</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Hit submit draft Akseptasi ketika nomor KTP sdh terdaftar sebelumnya</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t xml:space="preserve">[Test-Step 1] : Buka Postman
 [Test-Step 2] : Set request ke POST {{TESTING_API_GATEWAY}}/akseptasi/draft/submit 
@@ -2178,71 +2185,70 @@
 </t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095157-JCUEMP
 ktp: 0687495697403336
 </t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N26" s="3" t="inlineStr">
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
+      <c r="A27" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>TC-24</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Submit pengajuan dimana (Tanggal Realisasi - Tanggal Lahir) menghasilkan usia kurang dari batas minimum &gt; 18 tahun</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set POST {base_url}/akseptasi/draft/submit
@@ -2250,71 +2256,70 @@
 4. Hit Send</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095205-NVROFY
 ktp: 1725458943535859
 </t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L27" s="3" t="n"/>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N27" s="3" t="inlineStr">
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
+      <c r="A28" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>TC-25</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Submit pengajuan dimana kalkulasi (Realisasi - Lahir) menghasilkan usia tepat &gt; 18 tahun</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t xml:space="preserve">[Test_Step-1] : Buka Postman
 [Test_Step-2] : Set request ke POST {base_url}/akseptasi/draft/submit
@@ -2323,71 +2328,70 @@
 </t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095206-SWUPPG
 ktp: 7933509472397987
 </t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L28" s="3" t="n"/>
-      <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N28" s="3" t="inlineStr">
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
+      <c r="A29" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>TC-26</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Submit pengajuan dimana (Usia Riil saat Realisasi + Tenor) melebihi batas maksimal pengajuan 65 tahun (+ 1 hari)</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t xml:space="preserve">[Test_Step-1] : Buka Postman
 [Test_Step-2] : Set request ke POST {base_url}/akseptasi/draft/submit
@@ -2396,71 +2400,70 @@
 </t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095206-ELFQJA
 ktp: 8630458139439239
 </t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L29" s="3" t="n"/>
-      <c r="M29" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N29" s="3" t="inlineStr">
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
+      <c r="A30" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>TC-27</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Submit pengajuan dengan input parameter 'usia' fiktif/salah, namun Tanggal Lahir dan Realisasi menghasilkan usia yang valid  (usia pas 65 tahun)</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t xml:space="preserve">[Test_Step-1] : Buka Postman
 [Test_Step-2] : Set request ke POST {base_url}/akseptasi/draft/submit
@@ -2469,143 +2472,141 @@
 </t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095206-NUKGML
 ktp: 4201277434371275
 </t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L30" s="3" t="n"/>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N30" s="3" t="inlineStr">
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
+      <c r="A31" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>A8 - End to End Flow</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>TC-28</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Validasi End-to-End Generate E-Polis &amp; Cek ACS FMS</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>Sistem siap untuk memproses pengajuan asuransi dari awal (Submit Draft) hingga penerbitan E-Polis.</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>1. Buka halaman ACS &amp; FMS
 2. Cari nomor polis
 3. Verifikasi ketersediaan</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-095206-TMEZHX
 ktp: 6621997483706595
 </t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="L31" s="3" t="n"/>
-      <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N31" s="3" t="inlineStr">
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
+      <c r="A32" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>A8 - End to End Flow</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>TC-29</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Submit kembali Akseptasi setelah Batal (Data sama, Transaksi Beda)</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>Ada draft akseptasi yang sudah dibatalkan sebelumnya</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>1. Hit Submit Draft (Draft 1)
 2. Hit Inquiry Loan
@@ -2615,7 +2616,7 @@
 6. Hit Inquiry Loan ulang dengan Nomor Loan &amp; PK sama</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t xml:space="preserve">[DATA UTAMA]
 KTP: 6038990022059559
@@ -2629,70 +2630,69 @@
 </t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>Sistem mengizinkan reuse data (KTP, Loan, PK) selama pengajuan sebelumnya dibatalkan.</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="L32" s="3" t="n"/>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr">
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
+      <c r="A33" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>TC-30</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Submit Draft - Tenor panjang (15 thn) usia debitur muda (20 thn)</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>1. Set usia_debitur = 20
 2. Set tenor = 180 bulan
 3. Hit endpoint Submit Draft</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-093407-SRVUEE
 ktp: 3404387391812951
@@ -2701,423 +2701,417 @@
 </t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N33" s="3" t="inlineStr">
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
+      <c r="A34" t="n">
         <v>31</v>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>TC-31</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Submit Draft - Tenor panjang (15 thn) batas akhir usia tepat 65 thn</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>1. Set usia_debitur = 50
 2. Set tenor = 180 bulan
 3. Hit endpoint Submit Draft</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260810-102717-RWYFZM
-ktp: 5376576102555745
-nomor_loan: LN-048388
-</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
+      <c r="I34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260814-155028-BXHGYD
+ktp: 7930920405925650
+nomor_loan: LN-383173
+</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L34" s="3" t="n"/>
-      <c r="M34" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N34" s="3" t="inlineStr">
-        <is>
-          <t>10/08/2026</t>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n">
+      <c r="A35" t="n">
         <v>32</v>
       </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>TC-32</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Submit Draft - Tenor 6 thn dengan usia akhir 65 thn lebih sehari</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>1. Set tenor = 72 bulan
 2. Set usia akhir asuransi = 65 tahun + 1 hari
 3. Hit endpoint Submit Draft</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-100018-TNTREC
 ktp: 6359327397846375
 </t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
 3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="L35" s="3" t="n"/>
-      <c r="M35" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N35" s="3" t="inlineStr">
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n">
+      <c r="A36" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>TC-33</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Submit Draft - Usia 55 thn tenor 15 thn (Usia akhir &gt; 65)</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>1. Set usia = 55
 2. Set tenor = 180 bulan
 3. Hit endpoint Submit Draft</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-100019-GSUROR
 ktp: 2999787370638519
 </t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K36" s="3" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="L36" s="3" t="n"/>
-      <c r="M36" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N36" s="3" t="inlineStr">
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n">
+      <c r="A37" t="n">
         <v>34</v>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>TC-34</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Submit Draft - Inkosistensi logic tenor (10 thn) vs tgl akhir (5 thn)</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>1. Set tenor = 120 bulan
 2. Set tanggal_akhir = realisasi + 5 tahun
 3. Hit endpoint Submit Draft</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-100019-XVOYRS
 ktp: 0136768188684338
 </t>
         </is>
       </c>
-      <c r="J37" s="4" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K37" s="3" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="L37" s="3" t="n"/>
-      <c r="M37" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N37" s="3" t="inlineStr">
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n">
+      <c r="A38" t="n">
         <v>35</v>
       </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
         <is>
           <t>A2 - Submit Draft Akseptasi</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>TC-35</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Submit Draft - Inkosistensi logic tenor (2 thn) vs tgl akhir (10 thn)</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>Layanan Submit Draft (A2) beroperasi normal dan koneksi database stabil.</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>1. Set tenor = 24 bulan
 2. Set tanggal_akhir = realisasi + 10 tahun
 3. Hit endpoint Submit Draft</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t xml:space="preserve">nomor_transaksi: AKS-20260810-100019-DGMKFO
 ktp: 8318594002702523
 </t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
 2. Data tidak terecord atau termutasi di Database.</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="L38" s="3" t="n"/>
-      <c r="M38" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N38" s="3" t="inlineStr">
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n">
+      <c r="A39" t="n">
         <v>36</v>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Akseptasi H2H</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
         <is>
           <t>A1 - Kalkulasi Premi</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>TC-36</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Validasi Kalkulasi Premi dengan tenor &gt; 60 bulan (180 bulan) menggunakan rate maksimal (60 bulan = 0.725) dengan UP 100 Juta</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>Layanan Kalkulasi Premi (A1) beroperasi normal dan database stabil.</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>1. Buka Postman
 2. Set request ke POST {{TESTING_API_GATEWAY}}/kalkulator/premi
@@ -3125,39 +3119,388 @@
 4. Hit Send dan periksa respons rate &amp; premi</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t xml:space="preserve">ktp: 8217887972843606
 </t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>1. API berhasil memproses request (HTTP 200 OK).
 2. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
         </is>
       </c>
-      <c r="K39" s="3" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="L39" s="3" t="n"/>
-      <c r="M39" s="3" t="inlineStr">
-        <is>
-          <t>Fathur</t>
-        </is>
-      </c>
-      <c r="N39" s="3" t="inlineStr">
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Submit Draft Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>TC-37</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Submit Draft Akseptasi Multi Fasilitas Akumulasi &lt;= 500Jt</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>1. Generate KTP
+2. Submit Draft -&gt; Terbit Polis (UP 50 Juta)
+3. Set Payload Baru</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Draft dengan UP 450 Juta</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260814-140623-SLFSGB
+ktp: 3168900258421529
+</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Submit Draft Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>TC-38</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Submit Draft Akseptasi Multi Fasilitas Akumulasi &gt; 500Jt</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>1. Generate KTP
+2. Submit Draft -&gt; Terbit Polis (UP 50 Juta)
+3. Set Payload Baru</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Draft dengan UP 450 Juta 1 Rupiah</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260814-140832-KVISKL
+ktp: 7360359479212527
+</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>1. API menolak request dengan status gagal (400/422) dan mengembalikan pesan error validasi.
+2. Muncul pesan Error Limit CBC Accumulation.
+3. Data tidak terecord atau termutasi di Database.</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Kalkulator Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TC-39</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Simulasi Kalkulator Premi Multi Fasilitas Akumulasi &lt;= 500Jt</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>1. Generate KTP
+2. Submit Draft -&gt; Terbit Polis (UP 50 Juta)
+3. Set Payload Baru</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>1. Hit API Kalkulator Premi dengan UP 450 Juta</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ktp: 5144664616295173
+</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>1. API berhasil memproses simulasi kalkulasi dengan HTTP 200
+2. Total Akumulasi Valid
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Kalkulator Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TC-40</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Simulasi Kalkulator Premi Multi Fasilitas Akumulasi &gt; 500Jt</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>1. Generate KTP
+2. Submit Draft -&gt; Terbit Polis (UP 50 Juta)
+3. Set Payload Baru</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>1. Hit API Kalkulator Premi dengan UP 450 Juta 1 Rupiah</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ktp: 8840920497274831
+</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>1. API menolak request (HTTP 422).
+2. Muncul pesan Error Limit CBC Accumulation
+3. Data tidak terecord atau termutasi di Database.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Submit Draft Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>TC-41</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Submit Draft Akseptasi Multi Fasilitas (Fasilitas Pertama Tenor 180 Bulan) Akumulasi &lt;= 500Jt</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>1. Generate KTP
+2. Submit Draft dengan Tenor 180 Bulan -&gt; Terbit Polis (UP 50 Juta)
+3. Set Payload Baru</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Draft dengan UP 450 Juta</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260814-140846-BXWLLZ
+ktp: 4929626691647152
+</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>1. API berhasil memproses request (HTTP 200 OK).
+2. Field dinamis pada response (seperti nomor_transaksi, premi) ter-generate dengan format valid.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:N2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>